<commit_message>
pd sort of fixed kind of
</commit_message>
<xml_diff>
--- a/radar_design_output.xlsx
+++ b/radar_design_output.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="100" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="725" uniqueCount="25">
   <si>
     <t>param_names</t>
   </si>
@@ -502,7 +502,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="0">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
@@ -510,7 +510,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="0">
-        <v>0.75</v>
+        <v>0.29999999999999999</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
@@ -518,7 +518,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="0">
-        <v>0.75</v>
+        <v>0.29999999999999999</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
@@ -550,7 +550,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="0">
-        <v>0.099999999999999992</v>
+        <v>0.029999999999999999</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
@@ -596,7 +596,7 @@
         <v>14</v>
       </c>
       <c r="B2" s="0">
-        <v>4.2166024525176038</v>
+        <v>10.593355749341862</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
@@ -604,7 +604,7 @@
         <v>15</v>
       </c>
       <c r="B3" s="0">
-        <v>12316.782397935929</v>
+        <v>12229.184664940054</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
@@ -620,7 +620,7 @@
         <v>17</v>
       </c>
       <c r="B5" s="0">
-        <v>12435.862556378441</v>
+        <v>12526.930502651467</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
@@ -628,7 +628,7 @@
         <v>18</v>
       </c>
       <c r="B6" s="0">
-        <v>15</v>
+        <v>4.5</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
@@ -636,7 +636,7 @@
         <v>19</v>
       </c>
       <c r="B7" s="0">
-        <v>66.005290868074056</v>
+        <v>165.01322717018513</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
@@ -644,7 +644,7 @@
         <v>20</v>
       </c>
       <c r="B8" s="0">
-        <v>254.64790894703253</v>
+        <v>636.61977236758139</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
@@ -652,7 +652,7 @@
         <v>21</v>
       </c>
       <c r="B9" s="0">
-        <v>0.00085717400000000015</v>
+        <v>0.99999700199999997</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
@@ -660,7 +660,7 @@
         <v>22</v>
       </c>
       <c r="B10" s="0">
-        <v>-13.197978655936669</v>
+        <v>-2.8331150308342865</v>
       </c>
     </row>
     <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">

</xml_diff>